<commit_message>
updated the app to add a user upload section, addining a test public data folder to act as a place holder, finally adding the logo that has been present on shiny for months
</commit_message>
<xml_diff>
--- a/Data/Public_Data.xlsx
+++ b/Data/Public_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kincercrovetti/Desktop/Academics/LAB/FungAMR_project/Shiny/App-3/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B22110E3-A855-5E44-9BB6-80375C9C7B28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2A5750C-7202-8F47-BACE-D998C9ED81BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1360" yWindow="920" windowWidth="28040" windowHeight="17260" xr2:uid="{CADE24F5-32B4-A342-AAE7-C1566645882D}"/>
+    <workbookView xWindow="1360" yWindow="880" windowWidth="28040" windowHeight="17260" xr2:uid="{CADE24F5-32B4-A342-AAE7-C1566645882D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="18">
   <si>
     <t xml:space="preserve">Author </t>
   </si>
@@ -69,13 +69,37 @@
   </si>
   <si>
     <t>Citation</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>test 1</t>
+  </si>
+  <si>
+    <t>Iceland</t>
+  </si>
+  <si>
+    <t xml:space="preserve">test 1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> test 1</t>
+  </si>
+  <si>
+    <t>test 2</t>
+  </si>
+  <si>
+    <t>Clinical</t>
+  </si>
+  <si>
+    <t>Agricultural</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -89,6 +113,12 @@
       <color indexed="8"/>
       <name val="Helvetica Neue"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -471,7 +501,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{047C2799-72AB-394A-8EC5-88B407AE0E50}">
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
@@ -506,7 +536,72 @@
         <v>9</v>
       </c>
     </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2" t="s">
+        <v>11</v>
+      </c>
+      <c r="J2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
+        <v>15</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I3" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>